<commit_message>
Publish FHIR IG from 616fcc477a9fd9896f50f0be87931c29515c8eb9 616fcc477a9fd9896f50f0be87931c29515c8eb9
</commit_message>
<xml_diff>
--- a/CodeSystem-list-purpose.xlsx
+++ b/CodeSystem-list-purpose.xlsx
@@ -24,13 +24,13 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://hl7.no/fhir/ig/hackathon-attendance-registration-app/CodeSystem/list-purpose</t>
+    <t>https://hl7.no/fhir/ig/hackathon-check-in-app/CodeSystem/list-purpose</t>
   </si>
   <si>
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0</t>
+    <t>0.6.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-25T13:18:28+00:00</t>
+    <t>2026-10-29T07:06:30+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Publish FHIR IG from 026a4d6423b858d70244eea3b7c6b47ae37f7e1e 026a4d6423b858d70244eea3b7c6b47ae37f7e1e
</commit_message>
<xml_diff>
--- a/CodeSystem-list-purpose.xlsx
+++ b/CodeSystem-list-purpose.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.6.0</t>
+    <t>0.6.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-29T08:26:45+00:00</t>
+    <t>2026-10-29T09:23:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>